<commit_message>
Preserve crew owners across handoffs and bound reload clock checks
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V161.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V161.xlsx
@@ -117,8 +117,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV161Table11" displayName="AuditV161Table11" ref="A5:E18" totalsRowShown="0">
-  <autoFilter ref="A5:E18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV161Table11" displayName="AuditV161Table11" ref="A5:E19" totalsRowShown="0">
+  <autoFilter ref="A5:E19"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V158"/>
@@ -1946,88 +1946,88 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/save.js</t>
+          <t xml:space="preserve">src/npc-annex-circulation-v159.js</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ee15bc4a5df71e98c50cdbbf980d46c02d8e48c08ba74f6be84c2587eaa45718</t>
+          <t xml:space="preserve">5034808833beea323a3a3836c60cfeb40d5822575e085f0bead50d8826038f81</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">59d429c858402a26a7768e47e6520aff95f6b6f12668f8bb69430502c8952e5d</t>
+          <t xml:space="preserve">30ff9afe4985a2e9db880845521e3fb4e31a38304f97a0a7c12c3c5ba54ef493</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deux circuits natifs relient Idris entre le réacteur et la salle des machines du pont 3, et Leila entre le mess et la cuisine du pont 1. Les mêmes acteurs de 44 × 92 unités marchent sur le sol 624 jusqu’aux vraies portes appariées ; leur changement de repère se produit uniquement derrière les vantaux opaques entièrement fermés. Les deux faces du cadre cuisine sont agrandies uniformément pour contenir la silhouette native ; les plaques suivent le cadre réel avec dix pixels de dégagement. L’état borné conserve les phases à la reprise et réagit aux interruptions, aux passages occupés et aux dialogues natifs.</t>
+          <t xml:space="preserve">Le retour à la routine native recrée la population via la méthode virtuelle commune afin de préserver les propriétaires superposés des trois circuits, y compris un collègue à terre ou en récupération médicale.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-service-routes-v161.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">sw.js</t>
+          <t xml:space="preserve">src/save.js</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6d9706400fc34044d293a0d54c43396662de77c7e676bc8631df5b4ae287216b</t>
+          <t xml:space="preserve">ee15bc4a5df71e98c50cdbbf980d46c02d8e48c08ba74f6be84c2587eaa45718</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fd43d5989bde6df59643796d7a9c23fbfaa3e444bb07967f6d90b8cfba40b76d</t>
+          <t xml:space="preserve">59d429c858402a26a7768e47e6520aff95f6b6f12668f8bb69430502c8952e5d</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admet les cinq nouveaux modules natifs V161 dans le shell hors ligne et distingue le cache de continuation pour charger ensemble les fonctionnalités de campagne Forge, récit APC et circulation de service.</t>
+          <t xml:space="preserve">Deux circuits natifs relient Idris entre le réacteur et la salle des machines du pont 3, et Leila entre le mess et la cuisine du pont 1. Les mêmes acteurs de 44 × 92 unités marchent sur le sol 624 jusqu’aux vraies portes appariées ; leur changement de repère se produit uniquement derrière les vantaux opaques entièrement fermés. Les deux faces du cadre cuisine sont agrandies uniformément pour contenir la silhouette native ; les plaques suivent le cadre réel avec dix pixels de dégagement. L’état borné conserve les phases à la reprise et réagit aux interruptions, aux passages occupés et aux dialogues natifs.</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-audit-v143.mjs ; scripts/verify-forge-campaign-v161.mjs ; scripts/verify-campaign-convoy-story-v161.mjs ; scripts/verify-npc-service-routes-v161.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-service-routes-v161.mjs</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/apc-convoy-runtime-v121.js</t>
+          <t xml:space="preserve">sw.js</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V160</t>
+          <t xml:space="preserve">6d9706400fc34044d293a0d54c43396662de77c7e676bc8631df5b4ae287216b</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b1fa0c689763ca94ddb37b99020acedcd176d057b5d26f16ef24f9171c39a4a9</t>
+          <t xml:space="preserve">fd43d5989bde6df59643796d7a9c23fbfaa3e444bb07967f6d90b8cfba40b76d</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le départ APC développe cinq phases originales Tantalus avec un choix facultatif de lecture du blindage ou du parcours, conservé sans bonus économique. Sept jalons natifs alimentent la radio et le HUD APC est regroupé. Trois questions de retour lisent seulement le résultat terminal et le checkpoint de la même opération native ; les lectures bornées dans insertionState survivent à la sauvegarde normalisée, sans rejouer de paiement.</t>
+          <t xml:space="preserve">Admet les cinq nouveaux modules natifs V161 dans le shell hors ligne et distingue le cache de continuation pour charger ensemble les fonctionnalités de campagne Forge, récit APC et circulation de service.</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-convoy-story-v161.mjs</t>
+          <t xml:space="preserve">scripts/verify-audit-v143.mjs ; scripts/verify-forge-campaign-v161.mjs ; scripts/verify-campaign-convoy-story-v161.mjs ; scripts/verify-npc-service-routes-v161.mjs</t>
         </is>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/apc-course-v131.js</t>
+          <t xml:space="preserve">src/apc-convoy-runtime-v121.js</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a9b6fe7fa4ee899497baf590a0ce09c42258ca4bd39d78816a743c1ec145fd03</t>
+          <t xml:space="preserve">b1fa0c689763ca94ddb37b99020acedcd176d057b5d26f16ef24f9171c39a4a9</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
@@ -2054,7 +2054,7 @@
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-convoy-story-ui-v161.js</t>
+          <t xml:space="preserve">src/apc-course-v131.js</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e5dad2c548c7cf05584e88330538f0d606d330e99645e5a48fcef51d235e707c</t>
+          <t xml:space="preserve">a9b6fe7fa4ee899497baf590a0ce09c42258ca4bd39d78816a743c1ec145fd03</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
@@ -2081,7 +2081,7 @@
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-convoy-story-v161.js</t>
+          <t xml:space="preserve">src/campaign-convoy-story-ui-v161.js</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">17e3abceb4554a1223d4a456038d7664d42c44d5b96297285b73814678fc274e</t>
+          <t xml:space="preserve">e5dad2c548c7cf05584e88330538f0d606d330e99645e5a48fcef51d235e707c</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
@@ -2108,7 +2108,7 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/forge-campaign-ui-v161.js</t>
+          <t xml:space="preserve">src/campaign-convoy-story-v161.js</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
@@ -2118,24 +2118,24 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e9d82bc38f661260687e53affe1fb9c272ec7ec6906d645cb91034d6756ef01b</t>
+          <t xml:space="preserve">17e3abceb4554a1223d4a456038d7664d42c44d5b96297285b73814678fc274e</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Une campagne locale ordonnée conserve les documents figés de deux à seize projets Mission/Vaisseau. Seule la réussite native de l’étape exacte ouvre la suivante ; les objectifs et choix narratifs sont conservés dans le reçu. Le prochain départ reste explicite, la progression des étapes terminées survit au rechargement et les modifications ultérieures des projets source ne réécrivent pas leurs copies. Les écritures locales détectent les conflits entre onglets et préservent les données corrompues sans les écraser.</t>
+          <t xml:space="preserve">Le départ APC développe cinq phases originales Tantalus avec un choix facultatif de lecture du blindage ou du parcours, conservé sans bonus économique. Sept jalons natifs alimentent la radio et le HUD APC est regroupé. Trois questions de retour lisent seulement le résultat terminal et le checkpoint de la même opération native ; les lectures bornées dans insertionState survivent à la sauvegarde normalisée, sans rejouer de paiement.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-forge-campaign-v161.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-convoy-story-v161.mjs</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/forge-campaign-v161.js</t>
+          <t xml:space="preserve">src/forge-campaign-ui-v161.js</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0f7b6cd7f062d6b392d27befa55751a788959dcc00f01fc15c03c61ec967c12</t>
+          <t xml:space="preserve">e9d82bc38f661260687e53affe1fb9c272ec7ec6906d645cb91034d6756ef01b</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
@@ -2162,7 +2162,7 @@
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-destination-signage-runtime-v138.js</t>
+          <t xml:space="preserve">src/forge-campaign-v161.js</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
@@ -2172,42 +2172,69 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f9502b068c8c53932e403b4b512d562ea72c9f145e8bb5c904dc8f7ab9dfd428</t>
+          <t xml:space="preserve">a0f7b6cd7f062d6b392d27befa55751a788959dcc00f01fc15c03c61ec967c12</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les plaques des deux faces du passage cuisine suivent le vrai cadre de porte apparié uniformément agrandi et conservent dix pixels de dégagement, au lieu du gabarit historique fixe.</t>
+          <t xml:space="preserve">Une campagne locale ordonnée conserve les documents figés de deux à seize projets Mission/Vaisseau. Seule la réussite native de l’étape exacte ouvre la suivante ; les objectifs et choix narratifs sont conservés dans le reçu. Le prochain départ reste explicite, la progression des étapes terminées survit au rechargement et les modifications ultérieures des projets source ne réécrivent pas leurs copies. Les écritures locales détectent les conflits entre onglets et préservent les données corrompues sans les écraser.</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-hub-destination-signage-v138.mjs</t>
+          <t xml:space="preserve">scripts/verify-forge-campaign-v161.mjs</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/hub-destination-signage-runtime-v138.js</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V160</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f9502b068c8c53932e403b4b512d562ea72c9f145e8bb5c904dc8f7ab9dfd428</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les plaques des deux faces du passage cuisine suivent le vrai cadre de porte apparié uniformément agrandi et conservent dix pixels de dégagement, au lieu du gabarit historique fixe.</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-hub-destination-signage-v138.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">src/npc-service-routes-v161.js</t>
         </is>
       </c>
-      <c r="B18" s="0" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V160</t>
         </is>
       </c>
-      <c r="C18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4099be016856f1d21d476e7789bd6f33a53b84c8a5aa5ef4e2a6d7bb938e6652</t>
-        </is>
-      </c>
-      <c r="D18" s="0" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1571979e0dfe7d6bbad7e120aa1edae445099911909da0e7e3748e514674e189</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Deux circuits natifs relient Idris entre le réacteur et la salle des machines du pont 3, et Leila entre le mess et la cuisine du pont 1. Les mêmes acteurs de 44 × 92 unités marchent sur le sol 624 jusqu’aux vraies portes appariées ; leur changement de repère se produit uniquement derrière les vantaux opaques entièrement fermés. Les deux faces du cadre cuisine sont agrandies uniformément pour contenir la silhouette native ; les plaques suivent le cadre réel avec dix pixels de dégagement. L’état borné conserve les phases à la reprise et réagit aux interruptions, aux passages occupés et aux dialogues natifs.</t>
         </is>
       </c>
-      <c r="E18" s="0" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-npc-service-routes-v161.mjs</t>
         </is>
@@ -23367,12 +23394,12 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deux circuits natifs relient Idris entre le réacteur et la salle des machines du pont 3, et Leila entre le mess et la cuisine du pont 1. Les mêmes acteurs de 44 × 92 unités marchent sur le sol 624 jusqu’aux vraies portes appariées ; leur changement de repère se produit uniquement derrière les vantaux opaques entièrement fermés. Les deux faces du cadre cuisine sont agrandies uniformément pour contenir la silhouette native ; les plaques suivent le cadre réel avec dix pixels de dégagement. L’état borné conserve les phases à la reprise et réagit aux interruptions, aux passages occupés et aux dialogues natifs.</t>
+          <t xml:space="preserve">Deux circuits natifs relient Idris entre le réacteur et la salle des machines du pont 3, et Leila entre le mess et la cuisine du pont 1. Les mêmes acteurs de 44 × 92 unités marchent sur le sol 624 jusqu’aux vraies portes appariées ; leur changement de repère se produit uniquement derrière les vantaux opaques entièrement fermés. Les deux faces du cadre cuisine sont agrandies uniformément pour contenir la silhouette native ; les plaques suivent le cadre réel avec dix pixels de dégagement. Le retour aux routines natives respecte la composition des trois propriétaires de circuit pour conserver les autres acteurs à terre ou en récupération médicale. L’état borné conserve les phases à la reprise et réagit aux interruptions, aux passages occupés et aux dialogues natifs.</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-routes-v161.js ; src/save.js ; src/app.js ; src/hub-destination-signage-runtime-v138.js</t>
+          <t xml:space="preserve">src/npc-service-routes-v161.js ; src/save.js ; src/app.js ; src/hub-destination-signage-runtime-v138.js ; src/npc-annex-circulation-v159.js</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
@@ -28199,12 +28226,12 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-routes-v161.js ; src/save.js ; src/app.js ; src/hub-destination-signage-runtime-v138.js</t>
+          <t xml:space="preserve">src/npc-service-routes-v161.js ; src/save.js ; src/app.js ; src/hub-destination-signage-runtime-v138.js ; src/npc-annex-circulation-v159.js</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deux circuits natifs relient Idris entre le réacteur et la salle des machines du pont 3, et Leila entre le mess et la cuisine du pont 1. Les mêmes acteurs de 44 × 92 unités marchent sur le sol 624 jusqu’aux vraies portes appariées ; leur changement de repère se produit uniquement derrière les vantaux opaques entièrement fermés. Les deux faces du cadre cuisine sont agrandies uniformément pour contenir la silhouette native ; les plaques suivent le cadre réel avec dix pixels de dégagement. L’état borné conserve les phases à la reprise et réagit aux interruptions, aux passages occupés et aux dialogues natifs.</t>
+          <t xml:space="preserve">Deux circuits natifs relient Idris entre le réacteur et la salle des machines du pont 3, et Leila entre le mess et la cuisine du pont 1. Les mêmes acteurs de 44 × 92 unités marchent sur le sol 624 jusqu’aux vraies portes appariées ; leur changement de repère se produit uniquement derrière les vantaux opaques entièrement fermés. Les deux faces du cadre cuisine sont agrandies uniformément pour contenir la silhouette native ; les plaques suivent le cadre réel avec dix pixels de dégagement. Le retour aux routines natives respecte la composition des trois propriétaires de circuit pour conserver les autres acteurs à terre ou en récupération médicale. L’état borné conserve les phases à la reprise et réagit aux interruptions, aux passages occupés et aux dialogues natifs.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">

</xml_diff>